<commit_message>
Initial commit: Selenium Contact List Automation Framework with Allure reporting
</commit_message>
<xml_diff>
--- a/src/main/resources/testdata/Data.xlsx
+++ b/src/main/resources/testdata/Data.xlsx
@@ -10,9 +10,8 @@
     <sheet name="Login" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="SignUp" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="AddContact" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="AddContact1" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="UpdateContact" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="DeleteContact" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="UpdateContact" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="DeleteContact" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -418,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,12 +445,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1234567</t>
+          <t>wrongpassword</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
     </row>
@@ -463,29 +462,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>wrongpassword</t>
+          <t>1234567</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Fail</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>invalid@test.com</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>12345</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -500,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -543,7 +525,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>testuser20260207054803@test.com</t>
+          <t>newuser54321@test.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -554,33 +536,6 @@
       <c r="E2" t="inlineStr">
         <is>
           <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>User</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>m46328690@gmail.com</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>1234567</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Fail</t>
         </is>
       </c>
     </row>
@@ -595,7 +550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -719,115 +674,6 @@
       <c r="L2" t="inlineStr">
         <is>
           <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Muhammad</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Ali</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1995-06-15</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>ali@test.com</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>03001234567</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Main Boulevard</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Gulberg</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Lahore</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Punjab</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>54000</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Pakistan</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2000-01-01</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>invalid@test.com</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>1234567890</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Test Street</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Test City</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Test State</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>12345</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Test Country</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Fail</t>
         </is>
       </c>
     </row>
@@ -842,7 +688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -910,52 +756,52 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Faris</t>
+          <t>Faris Updated</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Hamza</t>
+          <t>Hamza Updated</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2003-04-25</t>
+          <t>2003-05-15</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>faris@gmail.com</t>
+          <t>faris.updated@gmail.com</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>03114593627</t>
+          <t>03229876543</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>College Road</t>
+          <t>Updated Street</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Near Lajna Chok</t>
+          <t>Near Updated Location</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Lahore</t>
+          <t>Islamabad</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Punjab</t>
+          <t>Islamabad Capital</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>34325</t>
+          <t>44000</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -966,115 +812,6 @@
       <c r="L2" t="inlineStr">
         <is>
           <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Muhammad</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Ali</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1995-06-15</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>ali@test.com</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>03001234567</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Main Boulevard</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Gulberg</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Lahore</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Punjab</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>54000</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Pakistan</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2000-01-01</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>invalid@test.com</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>1234567890</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Test Street</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Test City</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Test State</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>12345</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Test Country</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Fail</t>
         </is>
       </c>
     </row>
@@ -1089,7 +826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1105,51 +842,6 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Birthdate</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Phone</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Street1</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Street2</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>City</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>State/Province</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Postal Code</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Country</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
           <t>Expected Result</t>
         </is>
       </c>
@@ -1167,243 +859,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2003-05-30</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>faris.updated@gmail.com</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>03229876543</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>New Street Address</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Near Mall</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Karachi</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Sindh</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>75500</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Pakistan</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
           <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Ali</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Muhammad</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1995-08-20</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>ali.updated@test.com</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>03337654321</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Updated Boulevard</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Phase 2</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Islamabad</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>ICT</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>44000</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Pakistan</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2000-01-01</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>invalid@test.com</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>1234567890</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Test Street</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Test City</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Test State</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>12345</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Test Country</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Fail</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>First Name</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Last Name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Faris</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Hamza</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Muhammad</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Ali</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>NonExistent</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Contact</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Fail</t>
         </is>
       </c>
     </row>

</xml_diff>